<commit_message>
feat: expand Add Project form to 40+ fields
</commit_message>
<xml_diff>
--- a/src/THE PLAN TO ACHEIVE THE BEAST/Emaar_Properties_Enhanced_CORRECTED.xlsx
+++ b/src/THE PLAN TO ACHEIVE THE BEAST/Emaar_Properties_Enhanced_CORRECTED.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TAD\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TAD\emaar-dashboard\src\THE PLAN TO ACHEIVE THE BEAST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F9291D-6DE2-4B3A-BE7D-21B4A0A402F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C63B7D0-510F-4E83-8593-EDE6112EDCD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Analytics Dashboard" sheetId="1" r:id="rId1"/>
@@ -3744,20 +3744,36 @@
     </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="17" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="9" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3770,12 +3786,6 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3783,10 +3793,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3794,22 +3800,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="17" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="9" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="9" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5730,7 +5730,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.17574356459534984"/>
+          <c:y val="0.13470777109413104"/>
+          <c:w val="0.77913257932523283"/>
+          <c:h val="0.8077911902310374"/>
+        </c:manualLayout>
+      </c:layout>
       <c:barChart>
         <c:barDir val="bar"/>
         <c:grouping val="clustered"/>
@@ -6388,14 +6398,14 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>60960</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>43</xdr:row>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>426720</xdr:colOff>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>37800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6423,16 +6433,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>632460</xdr:colOff>
+      <xdr:row>85</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>187200</xdr:colOff>
-      <xdr:row>52</xdr:row>
-      <xdr:rowOff>135000</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>1021080</xdr:colOff>
+      <xdr:row>106</xdr:row>
+      <xdr:rowOff>81660</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6459,16 +6469,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>129540</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>581400</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>77760</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>2280</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6495,16 +6505,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>175680</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>975360</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>187200</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>78120</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>289560</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6765,40 +6775,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="97" t="s">
+      <c r="B1" s="95" t="s">
         <v>54</v>
       </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
     </row>
     <row r="2" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="99" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
     </row>
     <row r="4" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="88" t="s">
+      <c r="B4" s="91" t="s">
         <v>56</v>
       </c>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
-      <c r="G4" s="85"/>
-      <c r="H4" s="85"/>
-      <c r="I4" s="85"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
+      <c r="G4" s="89"/>
+      <c r="H4" s="89"/>
+      <c r="I4" s="89"/>
     </row>
     <row r="5" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
@@ -6879,12 +6889,12 @@
       </c>
     </row>
     <row r="9" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="89" t="s">
+      <c r="B9" s="97" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="85"/>
-      <c r="D9" s="85"/>
-      <c r="E9" s="85"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="89"/>
+      <c r="E9" s="89"/>
     </row>
     <row r="10" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
@@ -6975,12 +6985,12 @@
       </c>
     </row>
     <row r="23" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="91" t="s">
+      <c r="B23" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="C23" s="85"/>
-      <c r="D23" s="85"/>
-      <c r="E23" s="85"/>
+      <c r="C23" s="89"/>
+      <c r="D23" s="89"/>
+      <c r="E23" s="89"/>
     </row>
     <row r="24" spans="2:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="11" t="s">
@@ -7053,12 +7063,12 @@
       </c>
     </row>
     <row r="30" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="95" t="s">
+      <c r="B30" s="101" t="s">
         <v>103</v>
       </c>
-      <c r="C30" s="85"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="85"/>
+      <c r="C30" s="89"/>
+      <c r="D30" s="89"/>
+      <c r="E30" s="89"/>
     </row>
     <row r="31" spans="2:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="11" t="s">
@@ -7187,12 +7197,12 @@
       </c>
     </row>
     <row r="41" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="92" t="s">
+      <c r="B41" s="98" t="s">
         <v>130</v>
       </c>
-      <c r="C41" s="85"/>
-      <c r="D41" s="85"/>
-      <c r="E41" s="85"/>
+      <c r="C41" s="89"/>
+      <c r="D41" s="89"/>
+      <c r="E41" s="89"/>
     </row>
     <row r="42" spans="2:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="11" t="s">
@@ -7267,12 +7277,12 @@
       </c>
     </row>
     <row r="52" spans="2:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="94" t="s">
+      <c r="B52" s="100" t="s">
         <v>141</v>
       </c>
-      <c r="C52" s="85"/>
-      <c r="D52" s="85"/>
-      <c r="E52" s="85"/>
+      <c r="C52" s="89"/>
+      <c r="D52" s="89"/>
+      <c r="E52" s="89"/>
     </row>
     <row r="53" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="11" t="s">
@@ -7347,16 +7357,16 @@
       </c>
     </row>
     <row r="63" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="96" t="s">
+      <c r="B63" s="94" t="s">
         <v>144</v>
       </c>
-      <c r="C63" s="85"/>
-      <c r="D63" s="85"/>
-      <c r="E63" s="85"/>
-      <c r="F63" s="85"/>
-      <c r="G63" s="85"/>
-      <c r="H63" s="85"/>
-      <c r="I63" s="85"/>
+      <c r="C63" s="89"/>
+      <c r="D63" s="89"/>
+      <c r="E63" s="89"/>
+      <c r="F63" s="89"/>
+      <c r="G63" s="89"/>
+      <c r="H63" s="89"/>
+      <c r="I63" s="89"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -7396,31 +7406,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>781</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>782</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="91" t="s">
         <v>783</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
     </row>
     <row r="5" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
@@ -7727,28 +7737,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>850</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>851</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
     </row>
     <row r="3" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
@@ -8117,44 +8127,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="91" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
     </row>
     <row r="5" spans="1:4" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="87" t="s">
+      <c r="A5" s="109" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="85"/>
-      <c r="C5" s="85"/>
-      <c r="D5" s="85"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="89"/>
     </row>
     <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="89" t="s">
+      <c r="A7" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="85"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="85"/>
+      <c r="B7" s="89"/>
+      <c r="C7" s="89"/>
+      <c r="D7" s="89"/>
     </row>
     <row r="8" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
@@ -8255,12 +8265,12 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="86" t="s">
+      <c r="A17" s="108" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="85"/>
-      <c r="C17" s="85"/>
-      <c r="D17" s="85"/>
+      <c r="B17" s="89"/>
+      <c r="C17" s="89"/>
+      <c r="D17" s="89"/>
     </row>
     <row r="18" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="23" t="s">
@@ -8380,20 +8390,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>932</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>933</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
     </row>
     <row r="4" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
@@ -8690,106 +8700,106 @@
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="88" t="s">
+      <c r="A27" s="91" t="s">
         <v>986</v>
       </c>
-      <c r="B27" s="85"/>
-      <c r="C27" s="85"/>
-      <c r="D27" s="85"/>
+      <c r="B27" s="89"/>
+      <c r="C27" s="89"/>
+      <c r="D27" s="89"/>
     </row>
     <row r="28" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="24" t="s">
         <v>987</v>
       </c>
-      <c r="B28" s="109" t="s">
+      <c r="B28" s="113" t="s">
         <v>988</v>
       </c>
-      <c r="C28" s="107"/>
-      <c r="D28" s="108"/>
+      <c r="C28" s="111"/>
+      <c r="D28" s="112"/>
     </row>
     <row r="29" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="26" t="s">
         <v>989</v>
       </c>
-      <c r="B29" s="106" t="s">
+      <c r="B29" s="110" t="s">
         <v>990</v>
       </c>
-      <c r="C29" s="107"/>
-      <c r="D29" s="108"/>
+      <c r="C29" s="111"/>
+      <c r="D29" s="112"/>
     </row>
     <row r="30" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="24" t="s">
         <v>991</v>
       </c>
-      <c r="B30" s="109" t="s">
+      <c r="B30" s="113" t="s">
         <v>992</v>
       </c>
-      <c r="C30" s="107"/>
-      <c r="D30" s="108"/>
+      <c r="C30" s="111"/>
+      <c r="D30" s="112"/>
     </row>
     <row r="31" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="26" t="s">
         <v>993</v>
       </c>
-      <c r="B31" s="106" t="s">
+      <c r="B31" s="110" t="s">
         <v>994</v>
       </c>
-      <c r="C31" s="107"/>
-      <c r="D31" s="108"/>
+      <c r="C31" s="111"/>
+      <c r="D31" s="112"/>
     </row>
     <row r="32" spans="1:4" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="24" t="s">
         <v>995</v>
       </c>
-      <c r="B32" s="109" t="s">
+      <c r="B32" s="113" t="s">
         <v>996</v>
       </c>
-      <c r="C32" s="107"/>
-      <c r="D32" s="108"/>
+      <c r="C32" s="111"/>
+      <c r="D32" s="112"/>
     </row>
     <row r="33" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="26" t="s">
         <v>997</v>
       </c>
-      <c r="B33" s="106" t="s">
+      <c r="B33" s="110" t="s">
         <v>998</v>
       </c>
-      <c r="C33" s="107"/>
-      <c r="D33" s="108"/>
+      <c r="C33" s="111"/>
+      <c r="D33" s="112"/>
     </row>
     <row r="34" spans="1:4" ht="68.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="24" t="s">
         <v>999</v>
       </c>
-      <c r="B34" s="109" t="s">
+      <c r="B34" s="113" t="s">
         <v>1000</v>
       </c>
-      <c r="C34" s="107"/>
-      <c r="D34" s="108"/>
+      <c r="C34" s="111"/>
+      <c r="D34" s="112"/>
     </row>
     <row r="35" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="26" t="s">
         <v>1001</v>
       </c>
-      <c r="B35" s="106" t="s">
+      <c r="B35" s="110" t="s">
         <v>1002</v>
       </c>
-      <c r="C35" s="107"/>
-      <c r="D35" s="108"/>
+      <c r="C35" s="111"/>
+      <c r="D35" s="112"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B32:D32"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="B33:D33"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B28:D28"/>
-    <mergeCell ref="A27:D27"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B32:D32"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -8814,26 +8824,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="103" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="98" t="s">
+      <c r="A2" s="102" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
     </row>
     <row r="3" spans="1:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="76" t="s">
@@ -9586,34 +9596,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>227</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>228</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="91" t="s">
         <v>229</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
     </row>
     <row r="5" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
@@ -9848,14 +9858,14 @@
       </c>
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="89" t="s">
+      <c r="A36" s="97" t="s">
         <v>287</v>
       </c>
-      <c r="B36" s="85"/>
-      <c r="C36" s="85"/>
-      <c r="D36" s="85"/>
-      <c r="E36" s="85"/>
-      <c r="F36" s="85"/>
+      <c r="B36" s="89"/>
+      <c r="C36" s="89"/>
+      <c r="D36" s="89"/>
+      <c r="E36" s="89"/>
+      <c r="F36" s="89"/>
     </row>
     <row r="37" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="23" t="s">
@@ -10090,55 +10100,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>328</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
-      <c r="L1" s="85"/>
-      <c r="M1" s="85"/>
-      <c r="N1" s="85"/>
-      <c r="O1" s="85"/>
-      <c r="P1" s="85"/>
-      <c r="Q1" s="85"/>
-      <c r="R1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="89"/>
+      <c r="R1" s="89"/>
     </row>
     <row r="2" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>329</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="85"/>
-      <c r="K2" s="85"/>
-      <c r="L2" s="85"/>
-      <c r="M2" s="85"/>
-      <c r="N2" s="85"/>
-      <c r="O2" s="85"/>
-      <c r="P2" s="85"/>
-      <c r="Q2" s="85"/>
-      <c r="R2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="89"/>
+      <c r="L2" s="89"/>
+      <c r="M2" s="89"/>
+      <c r="N2" s="89"/>
+      <c r="O2" s="89"/>
+      <c r="P2" s="89"/>
+      <c r="Q2" s="89"/>
+      <c r="R2" s="89"/>
     </row>
     <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="100" t="s">
+      <c r="A3" s="104" t="s">
         <v>330</v>
       </c>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
       <c r="D3" s="31" t="s">
         <v>331</v>
       </c>
@@ -10163,7 +10173,7 @@
       <c r="K3" s="35" t="s">
         <v>337</v>
       </c>
-      <c r="L3" s="111"/>
+      <c r="L3" s="85"/>
     </row>
     <row r="4" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
@@ -10255,7 +10265,7 @@
       <c r="K5" s="37">
         <v>2200</v>
       </c>
-      <c r="L5" s="112">
+      <c r="L5" s="86">
         <f t="shared" ref="L5:L52" si="0">I5/J5</f>
         <v>2333.3333333333335</v>
       </c>
@@ -10312,7 +10322,7 @@
       <c r="K6" s="39">
         <v>1800</v>
       </c>
-      <c r="L6" s="113">
+      <c r="L6" s="87">
         <f t="shared" si="0"/>
         <v>1861.5384615384614</v>
       </c>
@@ -10369,7 +10379,7 @@
       <c r="K7" s="37">
         <v>2100</v>
       </c>
-      <c r="L7" s="112">
+      <c r="L7" s="86">
         <f t="shared" si="0"/>
         <v>2184.84</v>
       </c>
@@ -10426,7 +10436,7 @@
       <c r="K8" s="39">
         <v>2800</v>
       </c>
-      <c r="L8" s="113">
+      <c r="L8" s="87">
         <f t="shared" si="0"/>
         <v>3063.2088888888889</v>
       </c>
@@ -10483,7 +10493,7 @@
       <c r="K9" s="37">
         <v>2000</v>
       </c>
-      <c r="L9" s="112">
+      <c r="L9" s="86">
         <f t="shared" si="0"/>
         <v>2200</v>
       </c>
@@ -10540,7 +10550,7 @@
       <c r="K10" s="39">
         <v>2622</v>
       </c>
-      <c r="L10" s="113">
+      <c r="L10" s="87">
         <f t="shared" si="0"/>
         <v>2240.4490358126723</v>
       </c>
@@ -10597,7 +10607,7 @@
       <c r="K11" s="37">
         <v>2322</v>
       </c>
-      <c r="L11" s="112">
+      <c r="L11" s="86">
         <f t="shared" si="0"/>
         <v>3801.4682860998651</v>
       </c>
@@ -10654,7 +10664,7 @@
       <c r="K12" s="39">
         <v>2200</v>
       </c>
-      <c r="L12" s="113">
+      <c r="L12" s="87">
         <f t="shared" si="0"/>
         <v>2114.2857142857142</v>
       </c>
@@ -10711,7 +10721,7 @@
       <c r="K13" s="37">
         <v>2500</v>
       </c>
-      <c r="L13" s="112">
+      <c r="L13" s="86">
         <f t="shared" si="0"/>
         <v>2347.8506666666667</v>
       </c>
@@ -10768,7 +10778,7 @@
       <c r="K14" s="39">
         <v>2200</v>
       </c>
-      <c r="L14" s="110">
+      <c r="L14" s="84">
         <f t="shared" si="0"/>
         <v>2242.8571428571427</v>
       </c>
@@ -10825,7 +10835,7 @@
       <c r="K15" s="37">
         <v>2200</v>
       </c>
-      <c r="L15" s="112">
+      <c r="L15" s="86">
         <f t="shared" si="0"/>
         <v>2571.4285714285716</v>
       </c>
@@ -10882,7 +10892,7 @@
       <c r="K16" s="39">
         <v>2400</v>
       </c>
-      <c r="L16" s="113">
+      <c r="L16" s="87">
         <f t="shared" si="0"/>
         <v>2360</v>
       </c>
@@ -10939,7 +10949,7 @@
       <c r="K17" s="37">
         <v>2000</v>
       </c>
-      <c r="L17" s="112">
+      <c r="L17" s="86">
         <f t="shared" si="0"/>
         <v>2628.5714285714284</v>
       </c>
@@ -10996,7 +11006,7 @@
       <c r="K18" s="39">
         <v>2200</v>
       </c>
-      <c r="L18" s="113">
+      <c r="L18" s="87">
         <f t="shared" si="0"/>
         <v>2071.4285714285716</v>
       </c>
@@ -11053,7 +11063,7 @@
       <c r="K19" s="37">
         <v>2000</v>
       </c>
-      <c r="L19" s="110">
+      <c r="L19" s="84">
         <f t="shared" si="0"/>
         <v>2286.982857142857</v>
       </c>
@@ -11110,7 +11120,7 @@
       <c r="K20" s="39">
         <v>2200</v>
       </c>
-      <c r="L20" s="113">
+      <c r="L20" s="87">
         <f t="shared" si="0"/>
         <v>2142.8571428571427</v>
       </c>
@@ -11167,7 +11177,7 @@
       <c r="K21" s="37">
         <v>2800</v>
       </c>
-      <c r="L21" s="112">
+      <c r="L21" s="86">
         <f t="shared" si="0"/>
         <v>2567.6923076923076</v>
       </c>
@@ -11224,7 +11234,7 @@
       <c r="K22" s="39">
         <v>2600</v>
       </c>
-      <c r="L22" s="113">
+      <c r="L22" s="87">
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
@@ -11281,7 +11291,7 @@
       <c r="K23" s="37">
         <v>2800</v>
       </c>
-      <c r="L23" s="112">
+      <c r="L23" s="86">
         <f t="shared" si="0"/>
         <v>2768.7285714285713</v>
       </c>
@@ -11338,7 +11348,7 @@
       <c r="K24" s="39">
         <v>2200</v>
       </c>
-      <c r="L24" s="113">
+      <c r="L24" s="87">
         <f t="shared" si="0"/>
         <v>2592.6971428571428</v>
       </c>
@@ -11395,7 +11405,7 @@
       <c r="K25" s="37">
         <v>2200</v>
       </c>
-      <c r="L25" s="112">
+      <c r="L25" s="86">
         <f t="shared" si="0"/>
         <v>2585.7142857142858</v>
       </c>
@@ -11452,7 +11462,7 @@
       <c r="K26" s="39">
         <v>2200</v>
       </c>
-      <c r="L26" s="110">
+      <c r="L26" s="84">
         <f t="shared" si="0"/>
         <v>2728.5714285714284</v>
       </c>
@@ -11509,7 +11519,7 @@
       <c r="K27" s="37">
         <v>2200</v>
       </c>
-      <c r="L27" s="110">
+      <c r="L27" s="84">
         <f t="shared" si="0"/>
         <v>2557.1428571428573</v>
       </c>
@@ -11566,7 +11576,7 @@
       <c r="K28" s="39">
         <v>2200</v>
       </c>
-      <c r="L28" s="110">
+      <c r="L28" s="84">
         <f t="shared" si="0"/>
         <v>2571.4285714285716</v>
       </c>
@@ -11623,7 +11633,7 @@
       <c r="K29" s="37">
         <v>2200</v>
       </c>
-      <c r="L29" s="110">
+      <c r="L29" s="84">
         <f t="shared" si="0"/>
         <v>2657.1428571428573</v>
       </c>
@@ -11680,7 +11690,7 @@
       <c r="K30" s="39">
         <v>2500</v>
       </c>
-      <c r="L30" s="110">
+      <c r="L30" s="84">
         <f t="shared" si="0"/>
         <v>3835.5542857142859</v>
       </c>
@@ -11737,7 +11747,7 @@
       <c r="K31" s="37">
         <v>2200</v>
       </c>
-      <c r="L31" s="110">
+      <c r="L31" s="84">
         <f t="shared" si="0"/>
         <v>2591.2685714285712</v>
       </c>
@@ -11794,7 +11804,7 @@
       <c r="K32" s="39">
         <v>4500</v>
       </c>
-      <c r="L32" s="113">
+      <c r="L32" s="87">
         <f t="shared" si="0"/>
         <v>4375</v>
       </c>
@@ -11851,7 +11861,7 @@
       <c r="K33" s="37">
         <v>4000</v>
       </c>
-      <c r="L33" s="112">
+      <c r="L33" s="86">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
@@ -11908,7 +11918,7 @@
       <c r="K34" s="39">
         <v>3500</v>
       </c>
-      <c r="L34" s="113">
+      <c r="L34" s="87">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
@@ -11965,7 +11975,7 @@
       <c r="K35" s="37">
         <v>3500</v>
       </c>
-      <c r="L35" s="112">
+      <c r="L35" s="86">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
@@ -12022,7 +12032,7 @@
       <c r="K36" s="39">
         <v>4000</v>
       </c>
-      <c r="L36" s="113">
+      <c r="L36" s="87">
         <f t="shared" si="0"/>
         <v>4375</v>
       </c>
@@ -12079,7 +12089,7 @@
       <c r="K37" s="37">
         <v>1800</v>
       </c>
-      <c r="L37" s="112">
+      <c r="L37" s="86">
         <f t="shared" si="0"/>
         <v>1846.1538461538462</v>
       </c>
@@ -12136,7 +12146,7 @@
       <c r="K38" s="39">
         <v>2500</v>
       </c>
-      <c r="L38" s="110">
+      <c r="L38" s="84">
         <f t="shared" si="0"/>
         <v>1400</v>
       </c>
@@ -12193,7 +12203,7 @@
       <c r="K39" s="37">
         <v>1800</v>
       </c>
-      <c r="L39" s="110">
+      <c r="L39" s="84">
         <f t="shared" si="0"/>
         <v>2384.6153846153848</v>
       </c>
@@ -12250,7 +12260,7 @@
       <c r="K40" s="39">
         <v>10004</v>
       </c>
-      <c r="L40" s="110">
+      <c r="L40" s="84">
         <f t="shared" si="0"/>
         <v>1030.3030303030303</v>
       </c>
@@ -12307,7 +12317,7 @@
       <c r="K41" s="37">
         <v>2608</v>
       </c>
-      <c r="L41" s="112">
+      <c r="L41" s="86">
         <f t="shared" si="0"/>
         <v>757.93462813832309</v>
       </c>
@@ -12364,7 +12374,7 @@
       <c r="K42" s="39">
         <v>5115</v>
       </c>
-      <c r="L42" s="113">
+      <c r="L42" s="87">
         <f t="shared" si="0"/>
         <v>1923.337856173677</v>
       </c>
@@ -12421,7 +12431,7 @@
       <c r="K43" s="37">
         <v>2176</v>
       </c>
-      <c r="L43" s="112">
+      <c r="L43" s="86">
         <f t="shared" si="0"/>
         <v>1700.3676470588234</v>
       </c>
@@ -12478,7 +12488,7 @@
       <c r="K44" s="39">
         <v>2176</v>
       </c>
-      <c r="L44" s="113">
+      <c r="L44" s="87">
         <f t="shared" si="0"/>
         <v>1700.3676470588234</v>
       </c>
@@ -12535,7 +12545,7 @@
       <c r="K45" s="37">
         <v>5400</v>
       </c>
-      <c r="L45" s="110">
+      <c r="L45" s="84">
         <f t="shared" si="0"/>
         <v>2073.6842105263158</v>
       </c>
@@ -12592,7 +12602,7 @@
       <c r="K46" s="39">
         <v>5115</v>
       </c>
-      <c r="L46" s="110">
+      <c r="L46" s="84">
         <f t="shared" si="0"/>
         <v>2103.120759837178</v>
       </c>
@@ -12649,7 +12659,7 @@
       <c r="K47" s="37">
         <v>5115</v>
       </c>
-      <c r="L47" s="110">
+      <c r="L47" s="84">
         <f t="shared" si="0"/>
         <v>2103.120759837178</v>
       </c>
@@ -12706,7 +12716,7 @@
       <c r="K48" s="39">
         <v>2500</v>
       </c>
-      <c r="L48" s="110">
+      <c r="L48" s="84">
         <f t="shared" si="0"/>
         <v>3300</v>
       </c>
@@ -12763,7 +12773,7 @@
       <c r="K49" s="37">
         <v>3000</v>
       </c>
-      <c r="L49" s="112">
+      <c r="L49" s="86">
         <f t="shared" si="0"/>
         <v>3000</v>
       </c>
@@ -12820,7 +12830,7 @@
       <c r="K50" s="39">
         <v>12700</v>
       </c>
-      <c r="L50" s="113">
+      <c r="L50" s="87">
         <f t="shared" si="0"/>
         <v>1920.8333333333333</v>
       </c>
@@ -12877,7 +12887,7 @@
       <c r="K51" s="37">
         <v>3500</v>
       </c>
-      <c r="L51" s="110">
+      <c r="L51" s="84">
         <f t="shared" si="0"/>
         <v>3600</v>
       </c>
@@ -12934,7 +12944,7 @@
       <c r="K52" s="39">
         <v>3000</v>
       </c>
-      <c r="L52" s="113">
+      <c r="L52" s="87">
         <f t="shared" si="0"/>
         <v>1136.3636363636363</v>
       </c>
@@ -13036,28 +13046,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>457</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>458</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
     </row>
     <row r="3" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
@@ -13349,33 +13359,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>530</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>531</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="91" t="s">
         <v>532</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
     </row>
     <row r="5" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
@@ -13683,13 +13693,13 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="89" t="s">
+      <c r="A24" s="97" t="s">
         <v>543</v>
       </c>
-      <c r="B24" s="85"/>
-      <c r="C24" s="85"/>
-      <c r="D24" s="85"/>
-      <c r="E24" s="85"/>
+      <c r="B24" s="89"/>
+      <c r="C24" s="89"/>
+      <c r="D24" s="89"/>
+      <c r="E24" s="89"/>
     </row>
     <row r="25" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="23" t="s">
@@ -13885,28 +13895,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>583</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>584</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="88" t="s">
+      <c r="A4" s="91" t="s">
         <v>585</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
+      <c r="B4" s="89"/>
+      <c r="C4" s="89"/>
+      <c r="D4" s="89"/>
     </row>
     <row r="5" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
@@ -14063,12 +14073,12 @@
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="101" t="s">
+      <c r="A18" s="90" t="s">
         <v>627</v>
       </c>
-      <c r="B18" s="85"/>
-      <c r="C18" s="85"/>
-      <c r="D18" s="85"/>
+      <c r="B18" s="89"/>
+      <c r="C18" s="89"/>
+      <c r="D18" s="89"/>
     </row>
     <row r="19" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="23" t="s">
@@ -14155,12 +14165,12 @@
       </c>
     </row>
     <row r="26" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="102" t="s">
+      <c r="A26" s="92" t="s">
         <v>652</v>
       </c>
-      <c r="B26" s="85"/>
-      <c r="C26" s="85"/>
-      <c r="D26" s="85"/>
+      <c r="B26" s="89"/>
+      <c r="C26" s="89"/>
+      <c r="D26" s="89"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -14195,36 +14205,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>653</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>654</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
     </row>
     <row r="4" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="103" t="s">
+      <c r="A4" s="105" t="s">
         <v>655</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="104" t="s">
+      <c r="B4" s="89"/>
+      <c r="C4" s="106" t="s">
         <v>656</v>
       </c>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
+      <c r="D4" s="89"/>
+      <c r="E4" s="89"/>
+      <c r="F4" s="89"/>
     </row>
     <row r="6" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
@@ -14473,55 +14483,55 @@
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="26" customWidth="1"/>
+    <col min="10" max="10" width="33.88671875" customWidth="1"/>
     <col min="11" max="11" width="28" customWidth="1"/>
     <col min="27" max="27" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="33.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>696</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
     </row>
     <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="93" t="s">
         <v>697</v>
       </c>
-      <c r="B2" s="85"/>
-      <c r="C2" s="85"/>
-      <c r="D2" s="85"/>
-      <c r="E2" s="85"/>
-      <c r="F2" s="85"/>
-      <c r="G2" s="85"/>
-      <c r="H2" s="85"/>
-      <c r="I2" s="85"/>
-      <c r="J2" s="85"/>
-      <c r="K2" s="85"/>
+      <c r="B2" s="89"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="89"/>
+      <c r="E2" s="89"/>
+      <c r="F2" s="89"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="89"/>
     </row>
     <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="102" t="s">
+      <c r="A3" s="92" t="s">
         <v>698</v>
       </c>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="85"/>
+      <c r="B3" s="89"/>
+      <c r="C3" s="89"/>
+      <c r="D3" s="89"/>
+      <c r="E3" s="89"/>
+      <c r="F3" s="89"/>
+      <c r="G3" s="89"/>
+      <c r="H3" s="89"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
+      <c r="K3" s="89"/>
     </row>
     <row r="4" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
@@ -15636,139 +15646,139 @@
       <c r="K36" s="68"/>
     </row>
     <row r="38" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="100" t="s">
+      <c r="A38" s="104" t="s">
         <v>772</v>
       </c>
-      <c r="B38" s="85"/>
-      <c r="C38" s="85"/>
-      <c r="D38" s="85"/>
-      <c r="E38" s="85"/>
-      <c r="F38" s="85"/>
-      <c r="G38" s="85"/>
-      <c r="H38" s="85"/>
-      <c r="I38" s="85"/>
-      <c r="J38" s="85"/>
-      <c r="K38" s="85"/>
+      <c r="B38" s="89"/>
+      <c r="C38" s="89"/>
+      <c r="D38" s="89"/>
+      <c r="E38" s="89"/>
+      <c r="F38" s="89"/>
+      <c r="G38" s="89"/>
+      <c r="H38" s="89"/>
+      <c r="I38" s="89"/>
+      <c r="J38" s="89"/>
+      <c r="K38" s="89"/>
     </row>
     <row r="39" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="105" t="s">
+      <c r="A39" s="107" t="s">
         <v>773</v>
       </c>
-      <c r="B39" s="85"/>
-      <c r="C39" s="85"/>
-      <c r="D39" s="85"/>
-      <c r="E39" s="85"/>
-      <c r="F39" s="85"/>
-      <c r="G39" s="85"/>
-      <c r="H39" s="85"/>
-      <c r="I39" s="85"/>
-      <c r="J39" s="85"/>
-      <c r="K39" s="85"/>
+      <c r="B39" s="89"/>
+      <c r="C39" s="89"/>
+      <c r="D39" s="89"/>
+      <c r="E39" s="89"/>
+      <c r="F39" s="89"/>
+      <c r="G39" s="89"/>
+      <c r="H39" s="89"/>
+      <c r="I39" s="89"/>
+      <c r="J39" s="89"/>
+      <c r="K39" s="89"/>
     </row>
     <row r="40" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="105" t="s">
+      <c r="A40" s="107" t="s">
         <v>774</v>
       </c>
-      <c r="B40" s="85"/>
-      <c r="C40" s="85"/>
-      <c r="D40" s="85"/>
-      <c r="E40" s="85"/>
-      <c r="F40" s="85"/>
-      <c r="G40" s="85"/>
-      <c r="H40" s="85"/>
-      <c r="I40" s="85"/>
-      <c r="J40" s="85"/>
-      <c r="K40" s="85"/>
+      <c r="B40" s="89"/>
+      <c r="C40" s="89"/>
+      <c r="D40" s="89"/>
+      <c r="E40" s="89"/>
+      <c r="F40" s="89"/>
+      <c r="G40" s="89"/>
+      <c r="H40" s="89"/>
+      <c r="I40" s="89"/>
+      <c r="J40" s="89"/>
+      <c r="K40" s="89"/>
     </row>
     <row r="41" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="105" t="s">
+      <c r="A41" s="107" t="s">
         <v>775</v>
       </c>
-      <c r="B41" s="85"/>
-      <c r="C41" s="85"/>
-      <c r="D41" s="85"/>
-      <c r="E41" s="85"/>
-      <c r="F41" s="85"/>
-      <c r="G41" s="85"/>
-      <c r="H41" s="85"/>
-      <c r="I41" s="85"/>
-      <c r="J41" s="85"/>
-      <c r="K41" s="85"/>
+      <c r="B41" s="89"/>
+      <c r="C41" s="89"/>
+      <c r="D41" s="89"/>
+      <c r="E41" s="89"/>
+      <c r="F41" s="89"/>
+      <c r="G41" s="89"/>
+      <c r="H41" s="89"/>
+      <c r="I41" s="89"/>
+      <c r="J41" s="89"/>
+      <c r="K41" s="89"/>
     </row>
     <row r="42" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="105" t="s">
+      <c r="A42" s="107" t="s">
         <v>776</v>
       </c>
-      <c r="B42" s="85"/>
-      <c r="C42" s="85"/>
-      <c r="D42" s="85"/>
-      <c r="E42" s="85"/>
-      <c r="F42" s="85"/>
-      <c r="G42" s="85"/>
-      <c r="H42" s="85"/>
-      <c r="I42" s="85"/>
-      <c r="J42" s="85"/>
-      <c r="K42" s="85"/>
+      <c r="B42" s="89"/>
+      <c r="C42" s="89"/>
+      <c r="D42" s="89"/>
+      <c r="E42" s="89"/>
+      <c r="F42" s="89"/>
+      <c r="G42" s="89"/>
+      <c r="H42" s="89"/>
+      <c r="I42" s="89"/>
+      <c r="J42" s="89"/>
+      <c r="K42" s="89"/>
     </row>
     <row r="43" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="105" t="s">
+      <c r="A43" s="107" t="s">
         <v>777</v>
       </c>
-      <c r="B43" s="85"/>
-      <c r="C43" s="85"/>
-      <c r="D43" s="85"/>
-      <c r="E43" s="85"/>
-      <c r="F43" s="85"/>
-      <c r="G43" s="85"/>
-      <c r="H43" s="85"/>
-      <c r="I43" s="85"/>
-      <c r="J43" s="85"/>
-      <c r="K43" s="85"/>
+      <c r="B43" s="89"/>
+      <c r="C43" s="89"/>
+      <c r="D43" s="89"/>
+      <c r="E43" s="89"/>
+      <c r="F43" s="89"/>
+      <c r="G43" s="89"/>
+      <c r="H43" s="89"/>
+      <c r="I43" s="89"/>
+      <c r="J43" s="89"/>
+      <c r="K43" s="89"/>
     </row>
     <row r="44" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="105" t="s">
+      <c r="A44" s="107" t="s">
         <v>778</v>
       </c>
-      <c r="B44" s="85"/>
-      <c r="C44" s="85"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="85"/>
-      <c r="F44" s="85"/>
-      <c r="G44" s="85"/>
-      <c r="H44" s="85"/>
-      <c r="I44" s="85"/>
-      <c r="J44" s="85"/>
-      <c r="K44" s="85"/>
+      <c r="B44" s="89"/>
+      <c r="C44" s="89"/>
+      <c r="D44" s="89"/>
+      <c r="E44" s="89"/>
+      <c r="F44" s="89"/>
+      <c r="G44" s="89"/>
+      <c r="H44" s="89"/>
+      <c r="I44" s="89"/>
+      <c r="J44" s="89"/>
+      <c r="K44" s="89"/>
     </row>
     <row r="45" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="105" t="s">
+      <c r="A45" s="107" t="s">
         <v>779</v>
       </c>
-      <c r="B45" s="85"/>
-      <c r="C45" s="85"/>
-      <c r="D45" s="85"/>
-      <c r="E45" s="85"/>
-      <c r="F45" s="85"/>
-      <c r="G45" s="85"/>
-      <c r="H45" s="85"/>
-      <c r="I45" s="85"/>
-      <c r="J45" s="85"/>
-      <c r="K45" s="85"/>
+      <c r="B45" s="89"/>
+      <c r="C45" s="89"/>
+      <c r="D45" s="89"/>
+      <c r="E45" s="89"/>
+      <c r="F45" s="89"/>
+      <c r="G45" s="89"/>
+      <c r="H45" s="89"/>
+      <c r="I45" s="89"/>
+      <c r="J45" s="89"/>
+      <c r="K45" s="89"/>
     </row>
     <row r="46" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="105" t="s">
+      <c r="A46" s="107" t="s">
         <v>780</v>
       </c>
-      <c r="B46" s="85"/>
-      <c r="C46" s="85"/>
-      <c r="D46" s="85"/>
-      <c r="E46" s="85"/>
-      <c r="F46" s="85"/>
-      <c r="G46" s="85"/>
-      <c r="H46" s="85"/>
-      <c r="I46" s="85"/>
-      <c r="J46" s="85"/>
-      <c r="K46" s="85"/>
+      <c r="B46" s="89"/>
+      <c r="C46" s="89"/>
+      <c r="D46" s="89"/>
+      <c r="E46" s="89"/>
+      <c r="F46" s="89"/>
+      <c r="G46" s="89"/>
+      <c r="H46" s="89"/>
+      <c r="I46" s="89"/>
+      <c r="J46" s="89"/>
+      <c r="K46" s="89"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:K34" xr:uid="{00000000-0009-0000-0000-000008000000}"/>

</xml_diff>